<commit_message>
battle of labyrinth cover fix
</commit_message>
<xml_diff>
--- a/RIORDANVERSE.xlsx
+++ b/RIORDANVERSE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E43E77-AC69-4269-BFE9-0A0011F44B24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F5A6B7A-483B-4A13-A3F1-11BF60ABECE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -562,9 +562,6 @@
     <t>https://covers.openlibrary.org/b/id/15090302-L.jpg</t>
   </si>
   <si>
-    <t>https://covers.openlibrary.org/b/id/10082411-L.jpg</t>
-  </si>
-  <si>
     <t>https://openlibrary.org/books/OL26304391M/The_Battle_of_the_Labyrinth</t>
   </si>
   <si>
@@ -698,6 +695,9 @@
   </si>
   <si>
     <t>https://openlibrary.org/books/OL62135323M/Camp_Half-Blood_from_the_World_of_Percy_Jackson</t>
+  </si>
+  <si>
+    <t>https://covers.openlibrary.org/b/id/15250714-L.jpg</t>
   </si>
 </sst>
 </file>
@@ -1519,10 +1519,10 @@
         <v>17</v>
       </c>
       <c r="K11" t="s">
+        <v>223</v>
+      </c>
+      <c r="O11" t="s">
         <v>224</v>
-      </c>
-      <c r="O11" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -2220,10 +2220,10 @@
         <v>17</v>
       </c>
       <c r="K30" t="s">
+        <v>225</v>
+      </c>
+      <c r="O30" t="s">
         <v>180</v>
-      </c>
-      <c r="O30" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
@@ -2249,10 +2249,10 @@
         <v>17</v>
       </c>
       <c r="K31" t="s">
+        <v>181</v>
+      </c>
+      <c r="O31" t="s">
         <v>182</v>
-      </c>
-      <c r="O31" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
@@ -2278,10 +2278,10 @@
         <v>17</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O32" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
@@ -2307,10 +2307,10 @@
         <v>17</v>
       </c>
       <c r="K33" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O33" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
@@ -2336,10 +2336,10 @@
         <v>17</v>
       </c>
       <c r="K34" t="s">
+        <v>187</v>
+      </c>
+      <c r="O34" t="s">
         <v>188</v>
-      </c>
-      <c r="O34" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
@@ -2365,10 +2365,10 @@
         <v>17</v>
       </c>
       <c r="K35" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="O35" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
@@ -2394,10 +2394,10 @@
         <v>17</v>
       </c>
       <c r="K36" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O36" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
@@ -2423,10 +2423,10 @@
         <v>17</v>
       </c>
       <c r="K37" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="O37" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
@@ -2452,10 +2452,10 @@
         <v>17</v>
       </c>
       <c r="K38" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O38" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
@@ -2481,10 +2481,10 @@
         <v>17</v>
       </c>
       <c r="K39" t="s">
+        <v>201</v>
+      </c>
+      <c r="O39" t="s">
         <v>202</v>
-      </c>
-      <c r="O39" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
@@ -2510,10 +2510,10 @@
         <v>17</v>
       </c>
       <c r="K40" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O40" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
@@ -2539,10 +2539,10 @@
         <v>17</v>
       </c>
       <c r="K41" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O41" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
@@ -2568,10 +2568,10 @@
         <v>17</v>
       </c>
       <c r="K42" t="s">
+        <v>203</v>
+      </c>
+      <c r="O42" t="s">
         <v>204</v>
-      </c>
-      <c r="O42" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
@@ -2597,10 +2597,10 @@
         <v>17</v>
       </c>
       <c r="K43" t="s">
+        <v>205</v>
+      </c>
+      <c r="O43" t="s">
         <v>206</v>
-      </c>
-      <c r="O43" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
@@ -2626,10 +2626,10 @@
         <v>17</v>
       </c>
       <c r="K44" t="s">
+        <v>207</v>
+      </c>
+      <c r="O44" t="s">
         <v>208</v>
-      </c>
-      <c r="O44" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
@@ -2655,10 +2655,10 @@
         <v>17</v>
       </c>
       <c r="K45" t="s">
+        <v>209</v>
+      </c>
+      <c r="O45" t="s">
         <v>210</v>
-      </c>
-      <c r="O45" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
@@ -2684,10 +2684,10 @@
         <v>17</v>
       </c>
       <c r="K46" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="O46" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
@@ -2713,10 +2713,10 @@
         <v>17</v>
       </c>
       <c r="K47" t="s">
+        <v>213</v>
+      </c>
+      <c r="O47" t="s">
         <v>214</v>
-      </c>
-      <c r="O47" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
@@ -2742,10 +2742,10 @@
         <v>17</v>
       </c>
       <c r="K48" t="s">
+        <v>215</v>
+      </c>
+      <c r="O48" t="s">
         <v>216</v>
-      </c>
-      <c r="O48" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
@@ -2771,10 +2771,10 @@
         <v>17</v>
       </c>
       <c r="K49" t="s">
+        <v>217</v>
+      </c>
+      <c r="O49" t="s">
         <v>218</v>
-      </c>
-      <c r="O49" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
@@ -2800,10 +2800,10 @@
         <v>17</v>
       </c>
       <c r="K50" t="s">
+        <v>219</v>
+      </c>
+      <c r="O50" t="s">
         <v>220</v>
-      </c>
-      <c r="O50" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
@@ -2829,10 +2829,10 @@
         <v>17</v>
       </c>
       <c r="K51" t="s">
+        <v>221</v>
+      </c>
+      <c r="O51" t="s">
         <v>222</v>
-      </c>
-      <c r="O51" t="s">
-        <v>223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>